<commit_message>
Análise de estabilidade. Cálculo de Flash e Delta_G para múltiplas composições. Avaliação do menor Delta_G para escolha da composição que promove separação de fases.
</commit_message>
<xml_diff>
--- a/Código_Pré_Modificações_Fred/dados_experimentais.xlsx
+++ b/Código_Pré_Modificações_Fred/dados_experimentais.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vitor\OneDrive\Documentos\Vitor\Projetos\PycharmProjects\Projeto_TotalEnergies\Código_Pré_Modificações_Fred\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D5FFA92-C2DC-4444-B0F5-7874CA72DC8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC30955E-0E3E-4FEE-B21E-BE89E0251DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="12" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Yanes_P1" sheetId="4" r:id="rId1"/>
@@ -25,8 +25,9 @@
     <sheet name="Alves_BR3_5C" sheetId="16" r:id="rId10"/>
     <sheet name="Alves_BR3_25C" sheetId="17" r:id="rId11"/>
     <sheet name="Alves_BR3_50C" sheetId="18" r:id="rId12"/>
-    <sheet name="Tharanivasan_Lloydminster_1" sheetId="8" r:id="rId13"/>
-    <sheet name="Tharanivasan_Lloydminster_2" sheetId="9" r:id="rId14"/>
+    <sheet name="Tharanivasan_Lloydminster_hept" sheetId="8" r:id="rId13"/>
+    <sheet name="Tharanivasan_Lloydminster_pent" sheetId="9" r:id="rId14"/>
+    <sheet name="Tharanivasan_Lloydminster_heptM" sheetId="20" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="13">
   <si>
     <t>Saturados</t>
   </si>
@@ -94,11 +95,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.000000000"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="0.0000000"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -285,7 +287,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -362,10 +364,13 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2665,6 +2670,448 @@
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
                 <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FA3EA911-3789-42A7-568B-623D99FB5877}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8991600" y="161925"/>
+            <a:ext cx="6658904" cy="3334215"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln>
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing15.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>95249</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>86654</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="2" name="Agrupar 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8C10AC3F-B1BF-4859-8990-4072DF2DCCB5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="2244089" y="85725"/>
+          <a:ext cx="13402605" cy="5029200"/>
+          <a:chOff x="2247899" y="161925"/>
+          <a:chExt cx="13402605" cy="5238750"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:grpSp>
+        <xdr:nvGrpSpPr>
+          <xdr:cNvPr id="3" name="Agrupar 2">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{63B31CE4-67CF-C999-3B90-9D412EB91180}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvGrpSpPr/>
+        </xdr:nvGrpSpPr>
+        <xdr:grpSpPr>
+          <a:xfrm>
+            <a:off x="2247899" y="180975"/>
+            <a:ext cx="6562726" cy="2771775"/>
+            <a:chOff x="2247899" y="180975"/>
+            <a:chExt cx="6562726" cy="2781300"/>
+          </a:xfrm>
+        </xdr:grpSpPr>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="6" name="Imagem 5">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7A9D735A-D168-1177-1659-D6D0FCECF3C5}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1"/>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="2257424" y="180975"/>
+              <a:ext cx="6477904" cy="2086266"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:ln>
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="7" name="CaixaDeTexto 6">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AE5D2B50-D126-7B99-2D63-9ACD1C9F81C2}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="2247899" y="2343150"/>
+              <a:ext cx="6562726" cy="619125"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:schemeClr val="bg1">
+                <a:lumMod val="95000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln w="12700" cmpd="sng">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="dk1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="0"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="pt-BR" sz="1600"/>
+                <a:t>Dados de yields não disponíveis na tese</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="pt-BR" sz="1600" baseline="0"/>
+                <a:t> nem</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="pt-BR" sz="1600"/>
+                <a:t> no artigo de Akbarzadeh (2005 )</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </xdr:grpSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="4" name="CaixaDeTexto 3">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B849BE8-AEF1-1C25-3AE1-6E202F98E869}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="9134924" y="3590925"/>
+            <a:ext cx="6352725" cy="1809750"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="38100" cmpd="sng">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+              <a:spcBef>
+                <a:spcPts val="0"/>
+              </a:spcBef>
+              <a:spcAft>
+                <a:spcPts val="0"/>
+              </a:spcAft>
+              <a:buClrTx/>
+              <a:buSzTx/>
+              <a:buFontTx/>
+              <a:buNone/>
+              <a:tabLst/>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="pt-BR" sz="1400"/>
+              <a:t>As variáveis destacadas acima alimentam</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+              <a:t> o</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="pt-BR" sz="1400"/>
+              <a:t> arquivo</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+              <a:t>: </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="pt-BR" sz="1400">
+                <a:solidFill>
+                  <a:schemeClr val="dk1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>'variáveis_entrada_código.txt'</a:t>
+            </a:r>
+            <a:endParaRPr lang="pt-BR" sz="1400"/>
+          </a:p>
+          <a:p>
+            <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+              <a:spcBef>
+                <a:spcPts val="0"/>
+              </a:spcBef>
+              <a:spcAft>
+                <a:spcPts val="0"/>
+              </a:spcAft>
+              <a:buClrTx/>
+              <a:buSzTx/>
+              <a:buFontTx/>
+              <a:buNone/>
+              <a:tabLst/>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="pt-BR" sz="1400"/>
+              <a:t>n_agregados = 30</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+              <a:spcBef>
+                <a:spcPts val="0"/>
+              </a:spcBef>
+              <a:spcAft>
+                <a:spcPts val="0"/>
+              </a:spcAft>
+              <a:buClrTx/>
+              <a:buSzTx/>
+              <a:buFontTx/>
+              <a:buNone/>
+              <a:tabLst/>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="pt-BR" sz="1400"/>
+              <a:t>MWmin</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+              <a:t> = 1800</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+              <a:spcBef>
+                <a:spcPts val="0"/>
+              </a:spcBef>
+              <a:spcAft>
+                <a:spcPts val="0"/>
+              </a:spcAft>
+              <a:buClrTx/>
+              <a:buSzTx/>
+              <a:buFontTx/>
+              <a:buNone/>
+              <a:tabLst/>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+              <a:t>MWmax = 30000</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+              <a:spcBef>
+                <a:spcPts val="0"/>
+              </a:spcBef>
+              <a:spcAft>
+                <a:spcPts val="0"/>
+              </a:spcAft>
+              <a:buClrTx/>
+              <a:buSzTx/>
+              <a:buFontTx/>
+              <a:buNone/>
+              <a:tabLst/>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+              <a:t>alfa = 3.5 (Obs: embora o Tharanivasan chame </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="pt-BR" sz="1400" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="dk1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>de </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="el-GR" sz="1400" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="dk1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>β</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="pt-BR" sz="1400" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="dk1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>, no nosso código o fator de forma da distribuição Gamma é a variável 'alfa'.)</a:t>
+            </a:r>
+            <a:br>
+              <a:rPr lang="pt-BR" sz="1400" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="dk1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+            </a:br>
+            <a:r>
+              <a:rPr lang="pt-BR" sz="1400" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="dk1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>MWavg = 3620.</a:t>
+            </a:r>
+            <a:endParaRPr lang="pt-BR" sz="1400">
+              <a:effectLst/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="5" name="Imagem 4">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{816FA57E-8AD0-F35D-5399-72836AF2C650}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -6405,13 +6852,13 @@
       <c r="B19" s="19"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B35" s="25"/>
@@ -6572,13 +7019,13 @@
       <c r="B19" s="19"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6716,13 +7163,13 @@
       </c>
     </row>
     <row r="20" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B35" s="25"/>
@@ -6743,7 +7190,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8D94E3C-228A-404B-AAAA-84368A7243B9}">
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="15.6640625" style="1" customWidth="1"/>
@@ -6815,358 +7262,216 @@
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="16">
-        <v>0.52</v>
-      </c>
-      <c r="B9" s="17">
-        <v>0</v>
+      <c r="A9" s="27">
+        <v>0.50725668750098696</v>
+      </c>
+      <c r="B9" s="27">
+        <v>3.2786886612808999E-3</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="16">
-        <v>0.53</v>
-      </c>
-      <c r="B10" s="17">
-        <v>0</v>
+      <c r="A10" s="27">
+        <v>0.53805307870333796</v>
+      </c>
+      <c r="B10" s="27">
+        <v>5.2458968551676198E-3</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="16">
-        <v>0.54</v>
-      </c>
-      <c r="B11" s="17">
-        <v>0</v>
+      <c r="A11" s="27">
+        <v>0.57840708796312601</v>
+      </c>
+      <c r="B11" s="27">
+        <v>2.2622919244106199E-2</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="16">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="B12" s="17">
-        <v>0</v>
+      <c r="A12" s="27">
+        <v>0.67185843518573596</v>
+      </c>
+      <c r="B12" s="27">
+        <v>6.7868845282751306E-2</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="16">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="B13" s="17">
-        <v>0</v>
+      <c r="A13" s="27">
+        <v>0.70371683796342999</v>
+      </c>
+      <c r="B13" s="27">
+        <v>8.0655736064628794E-2</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" s="16">
-        <v>0.57000000000000006</v>
-      </c>
-      <c r="B14" s="17">
-        <v>0</v>
+      <c r="A14" s="27">
+        <v>0.73345129861054503</v>
+      </c>
+      <c r="B14" s="27">
+        <v>9.4426230943449693E-2</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="16">
-        <v>0.58000000000000007</v>
-      </c>
-      <c r="B15" s="17">
-        <v>0</v>
+      <c r="A15" s="27">
+        <v>0.77380530787033297</v>
+      </c>
+      <c r="B15" s="27">
+        <v>0.10163933599250401</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="16">
-        <v>0.59000000000000008</v>
-      </c>
-      <c r="B16" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="16">
-        <v>0.60000000000000009</v>
-      </c>
-      <c r="B17" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="16">
-        <v>0.6100000000000001</v>
-      </c>
-      <c r="B18" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="16">
-        <v>0.62000000000000011</v>
-      </c>
-      <c r="B19" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="16">
-        <v>0.63000000000000012</v>
-      </c>
-      <c r="B20" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="16">
-        <v>0.64000000000000012</v>
-      </c>
-      <c r="B21" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="16">
-        <v>0.65000000000000013</v>
-      </c>
-      <c r="B22" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="16">
-        <v>0.66000000000000014</v>
-      </c>
-      <c r="B23" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="16">
-        <v>0.67000000000000015</v>
-      </c>
-      <c r="B24" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" s="16">
-        <v>0.68000000000000016</v>
-      </c>
-      <c r="B25" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="16">
-        <v>0.69000000000000017</v>
-      </c>
-      <c r="B26" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="16">
-        <v>0.70000000000000018</v>
-      </c>
-      <c r="B27" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" s="16">
-        <v>0.71000000000000019</v>
-      </c>
-      <c r="B28" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" s="16">
-        <v>0.7200000000000002</v>
-      </c>
-      <c r="B29" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" s="16">
-        <v>0.7300000000000002</v>
-      </c>
-      <c r="B30" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" s="16">
-        <v>0.74000000000000021</v>
-      </c>
-      <c r="B31" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A32" s="16">
-        <v>0.75000000000000022</v>
-      </c>
-      <c r="B32" s="17">
-        <v>0</v>
-      </c>
+      <c r="A16" s="27">
+        <v>0.87256630786911804</v>
+      </c>
+      <c r="B16" s="27">
+        <v>0.12327868866128</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="27">
+        <v>0.93203539120356504</v>
+      </c>
+      <c r="B17" s="27">
+        <v>0.123606558778129</v>
+      </c>
+      <c r="D17" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="27">
+        <v>0.95433625694392898</v>
+      </c>
+      <c r="B18" s="27">
+        <v>0.129508183359789</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" s="16"/>
+      <c r="B23" s="17"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" s="16"/>
+      <c r="B24" s="17"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" s="16"/>
+      <c r="B25" s="17"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26" s="16"/>
+      <c r="B26" s="17"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" s="16"/>
+      <c r="B27" s="17"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" s="16"/>
+      <c r="B28" s="17"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29" s="16"/>
+      <c r="B29" s="17"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" s="16"/>
+      <c r="B30" s="17"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" s="16"/>
+      <c r="B31" s="17"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32" s="16"/>
+      <c r="B32" s="17"/>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" s="16">
-        <v>0.76000000000000023</v>
-      </c>
-      <c r="B33" s="17">
-        <v>0</v>
-      </c>
+      <c r="A33" s="16"/>
+      <c r="B33" s="17"/>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" s="16">
-        <v>0.77000000000000024</v>
-      </c>
-      <c r="B34" s="17">
-        <v>0</v>
-      </c>
+      <c r="A34" s="16"/>
+      <c r="B34" s="17"/>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" s="16">
-        <v>0.78000000000000025</v>
-      </c>
-      <c r="B35" s="17">
-        <v>0</v>
-      </c>
+      <c r="A35" s="16"/>
+      <c r="B35" s="17"/>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" s="16">
-        <v>0.79000000000000026</v>
-      </c>
-      <c r="B36" s="17">
-        <v>0</v>
-      </c>
+      <c r="A36" s="16"/>
+      <c r="B36" s="17"/>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" s="16">
-        <v>0.80000000000000027</v>
-      </c>
-      <c r="B37" s="17">
-        <v>0</v>
-      </c>
+      <c r="A37" s="16"/>
+      <c r="B37" s="17"/>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" s="16">
-        <v>0.81000000000000028</v>
-      </c>
-      <c r="B38" s="17">
-        <v>0</v>
-      </c>
+      <c r="A38" s="16"/>
+      <c r="B38" s="17"/>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" s="16">
-        <v>0.82000000000000028</v>
-      </c>
-      <c r="B39" s="17">
-        <v>0</v>
-      </c>
+      <c r="A39" s="16"/>
+      <c r="B39" s="17"/>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40" s="16">
-        <v>0.83000000000000029</v>
-      </c>
-      <c r="B40" s="17">
-        <v>0</v>
-      </c>
+      <c r="A40" s="16"/>
+      <c r="B40" s="17"/>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" s="16">
-        <v>0.8400000000000003</v>
-      </c>
-      <c r="B41" s="17">
-        <v>0</v>
-      </c>
+      <c r="A41" s="16"/>
+      <c r="B41" s="17"/>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" s="16">
-        <v>0.85000000000000031</v>
-      </c>
-      <c r="B42" s="17">
-        <v>0</v>
-      </c>
+      <c r="A42" s="16"/>
+      <c r="B42" s="17"/>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43" s="16">
-        <v>0.86000000000000032</v>
-      </c>
-      <c r="B43" s="17">
-        <v>0</v>
-      </c>
+      <c r="A43" s="16"/>
+      <c r="B43" s="17"/>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44" s="16">
-        <v>0.87000000000000033</v>
-      </c>
-      <c r="B44" s="17">
-        <v>0</v>
-      </c>
+      <c r="A44" s="16"/>
+      <c r="B44" s="17"/>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" s="16">
-        <v>0.88000000000000034</v>
-      </c>
-      <c r="B45" s="17">
-        <v>0</v>
-      </c>
+      <c r="A45" s="16"/>
+      <c r="B45" s="17"/>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" s="16">
-        <v>0.89000000000000035</v>
-      </c>
-      <c r="B46" s="17">
-        <v>0</v>
-      </c>
+      <c r="A46" s="16"/>
+      <c r="B46" s="17"/>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" s="16">
-        <v>0.90000000000000036</v>
-      </c>
-      <c r="B47" s="17">
-        <v>0</v>
-      </c>
+      <c r="A47" s="16"/>
+      <c r="B47" s="17"/>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" s="16">
-        <v>0.91000000000000036</v>
-      </c>
-      <c r="B48" s="17">
-        <v>0</v>
-      </c>
+      <c r="A48" s="16"/>
+      <c r="B48" s="17"/>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" s="16">
-        <v>0.92000000000000037</v>
-      </c>
-      <c r="B49" s="17">
-        <v>0</v>
-      </c>
+      <c r="A49" s="16"/>
+      <c r="B49" s="17"/>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" s="16">
-        <v>0.93000000000000038</v>
-      </c>
-      <c r="B50" s="17">
-        <v>0</v>
-      </c>
+      <c r="A50" s="16"/>
+      <c r="B50" s="17"/>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" s="16">
-        <v>0.94000000000000039</v>
-      </c>
-      <c r="B51" s="17">
-        <v>0</v>
-      </c>
+      <c r="A51" s="16"/>
+      <c r="B51" s="17"/>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" s="16">
-        <v>0.9500000000000004</v>
-      </c>
-      <c r="B52" s="17">
-        <v>0</v>
-      </c>
+      <c r="A52" s="16"/>
+      <c r="B52" s="17"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D17:H17"/>
+  </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7" xr:uid="{2A74D785-ECF9-41EC-83E7-D06BFD039F5C}">
       <formula1>"n-heptano, n-pentano"</formula1>
@@ -7180,7 +7485,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E17C7ABB-BD74-4BD8-89A4-BE9C8A53E418}">
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="15.6640625" style="1" customWidth="1"/>
@@ -7251,422 +7556,268 @@
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="16">
-        <v>0.44</v>
-      </c>
-      <c r="B9" s="17">
-        <v>0</v>
+      <c r="A9" s="27">
+        <v>0.44778760416654001</v>
+      </c>
+      <c r="B9" s="27">
+        <v>9.8360534766381204E-3</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="16">
-        <v>0.45</v>
-      </c>
-      <c r="B10" s="17">
-        <v>0</v>
+      <c r="A10" s="27">
+        <v>0.48389381018527999</v>
+      </c>
+      <c r="B10" s="27">
+        <v>3.77049070975259E-2</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="16">
-        <v>0.46</v>
-      </c>
-      <c r="B11" s="17">
-        <v>0</v>
+      <c r="A11" s="27">
+        <v>0.51469028240773895</v>
+      </c>
+      <c r="B11" s="27">
+        <v>7.0819670080786101E-2</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="16">
-        <v>0.47000000000000003</v>
-      </c>
-      <c r="B12" s="17">
-        <v>0</v>
+      <c r="A12" s="27">
+        <v>0.555044291667527</v>
+      </c>
+      <c r="B12" s="27">
+        <v>9.77049196047306E-2</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="16">
-        <v>0.48000000000000004</v>
-      </c>
-      <c r="B13" s="17">
-        <v>0</v>
+      <c r="A13" s="27">
+        <v>0.65061950000060698</v>
+      </c>
+      <c r="B13" s="27">
+        <v>0.14196721027841999</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" s="16">
-        <v>0.49000000000000005</v>
-      </c>
-      <c r="B14" s="17">
-        <v>0</v>
+      <c r="A14" s="27">
+        <v>0.68460176388877003</v>
+      </c>
+      <c r="B14" s="27">
+        <v>0.15311475047605499</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="16">
-        <v>0.5</v>
-      </c>
-      <c r="B15" s="17">
-        <v>0</v>
+      <c r="A15" s="27">
+        <v>0.71327429398065101</v>
+      </c>
+      <c r="B15" s="27">
+        <v>0.15442623094344901</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="16">
-        <v>0.51</v>
-      </c>
-      <c r="B16" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="16">
-        <v>0.52</v>
-      </c>
-      <c r="B17" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="16">
-        <v>0.53</v>
-      </c>
-      <c r="B18" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="16">
-        <v>0.54</v>
-      </c>
-      <c r="B19" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="16">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="B20" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="16">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="B21" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="16">
-        <v>0.57000000000000006</v>
-      </c>
-      <c r="B22" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="16">
-        <v>0.58000000000000007</v>
-      </c>
-      <c r="B23" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="16">
-        <v>0.59000000000000008</v>
-      </c>
-      <c r="B24" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" s="16">
-        <v>0.60000000000000009</v>
-      </c>
-      <c r="B25" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="16">
-        <v>0.6100000000000001</v>
-      </c>
-      <c r="B26" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="16">
-        <v>0.62000000000000011</v>
-      </c>
-      <c r="B27" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" s="16">
-        <v>0.63000000000000012</v>
-      </c>
-      <c r="B28" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" s="16">
-        <v>0.64000000000000012</v>
-      </c>
-      <c r="B29" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" s="16">
-        <v>0.65000000000000013</v>
-      </c>
-      <c r="B30" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" s="16">
-        <v>0.66000000000000014</v>
-      </c>
-      <c r="B31" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A32" s="16">
-        <v>0.67000000000000015</v>
-      </c>
-      <c r="B32" s="17">
-        <v>0</v>
-      </c>
+      <c r="A16" s="27">
+        <v>0.75575216435090897</v>
+      </c>
+      <c r="B16" s="27">
+        <v>0.15999999791546499</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="27">
+        <v>0.86088490972131904</v>
+      </c>
+      <c r="B17" s="27">
+        <v>0.15704917937103299</v>
+      </c>
+      <c r="D17" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="27">
+        <v>0.92460171527670498</v>
+      </c>
+      <c r="B18" s="27">
+        <v>0.15999999791546499</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="27">
+        <v>0.94796459259241195</v>
+      </c>
+      <c r="B19" s="27">
+        <v>0.154754094806695</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="16"/>
+      <c r="B20" s="17"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="16"/>
+      <c r="B21" s="17"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" s="16"/>
+      <c r="B22" s="17"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" s="16"/>
+      <c r="B23" s="17"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" s="16"/>
+      <c r="B24" s="17"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" s="16"/>
+      <c r="B25" s="17"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26" s="16"/>
+      <c r="B26" s="17"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" s="16"/>
+      <c r="B27" s="17"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" s="16"/>
+      <c r="B28" s="17"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29" s="16"/>
+      <c r="B29" s="17"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" s="16"/>
+      <c r="B30" s="17"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" s="16"/>
+      <c r="B31" s="17"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32" s="16"/>
+      <c r="B32" s="17"/>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" s="16">
-        <v>0.68000000000000016</v>
-      </c>
-      <c r="B33" s="17">
-        <v>0</v>
-      </c>
+      <c r="A33" s="16"/>
+      <c r="B33" s="17"/>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" s="16">
-        <v>0.69000000000000017</v>
-      </c>
-      <c r="B34" s="17">
-        <v>0</v>
-      </c>
+      <c r="A34" s="16"/>
+      <c r="B34" s="17"/>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" s="16">
-        <v>0.70000000000000018</v>
-      </c>
-      <c r="B35" s="17">
-        <v>0</v>
-      </c>
+      <c r="A35" s="16"/>
+      <c r="B35" s="17"/>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" s="16">
-        <v>0.71000000000000019</v>
-      </c>
-      <c r="B36" s="17">
-        <v>0</v>
-      </c>
+      <c r="A36" s="16"/>
+      <c r="B36" s="17"/>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" s="16">
-        <v>0.7200000000000002</v>
-      </c>
-      <c r="B37" s="17">
-        <v>0</v>
-      </c>
+      <c r="A37" s="16"/>
+      <c r="B37" s="17"/>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" s="16">
-        <v>0.7300000000000002</v>
-      </c>
-      <c r="B38" s="17">
-        <v>0</v>
-      </c>
+      <c r="A38" s="16"/>
+      <c r="B38" s="17"/>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" s="16">
-        <v>0.74000000000000021</v>
-      </c>
-      <c r="B39" s="17">
-        <v>0</v>
-      </c>
+      <c r="A39" s="16"/>
+      <c r="B39" s="17"/>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40" s="16">
-        <v>0.75000000000000022</v>
-      </c>
-      <c r="B40" s="17">
-        <v>0</v>
-      </c>
+      <c r="A40" s="16"/>
+      <c r="B40" s="17"/>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" s="16">
-        <v>0.76000000000000023</v>
-      </c>
-      <c r="B41" s="17">
-        <v>0</v>
-      </c>
+      <c r="A41" s="16"/>
+      <c r="B41" s="17"/>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" s="16">
-        <v>0.77000000000000024</v>
-      </c>
-      <c r="B42" s="17">
-        <v>0</v>
-      </c>
+      <c r="A42" s="16"/>
+      <c r="B42" s="17"/>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43" s="16">
-        <v>0.78000000000000025</v>
-      </c>
-      <c r="B43" s="17">
-        <v>0</v>
-      </c>
+      <c r="A43" s="16"/>
+      <c r="B43" s="17"/>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44" s="16">
-        <v>0.79000000000000026</v>
-      </c>
-      <c r="B44" s="17">
-        <v>0</v>
-      </c>
+      <c r="A44" s="16"/>
+      <c r="B44" s="17"/>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" s="16">
-        <v>0.80000000000000027</v>
-      </c>
-      <c r="B45" s="17">
-        <v>0</v>
-      </c>
+      <c r="A45" s="16"/>
+      <c r="B45" s="17"/>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" s="16">
-        <v>0.81000000000000028</v>
-      </c>
-      <c r="B46" s="17">
-        <v>0</v>
-      </c>
+      <c r="A46" s="16"/>
+      <c r="B46" s="17"/>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" s="16">
-        <v>0.82000000000000028</v>
-      </c>
-      <c r="B47" s="17">
-        <v>0</v>
-      </c>
+      <c r="A47" s="16"/>
+      <c r="B47" s="17"/>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" s="16">
-        <v>0.83000000000000029</v>
-      </c>
-      <c r="B48" s="17">
-        <v>0</v>
-      </c>
+      <c r="A48" s="16"/>
+      <c r="B48" s="17"/>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" s="16">
-        <v>0.8400000000000003</v>
-      </c>
-      <c r="B49" s="17">
-        <v>0</v>
-      </c>
+      <c r="A49" s="16"/>
+      <c r="B49" s="17"/>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" s="16">
-        <v>0.85000000000000031</v>
-      </c>
-      <c r="B50" s="17">
-        <v>0</v>
-      </c>
+      <c r="A50" s="16"/>
+      <c r="B50" s="17"/>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" s="16">
-        <v>0.86000000000000032</v>
-      </c>
-      <c r="B51" s="17">
-        <v>0</v>
-      </c>
+      <c r="A51" s="16"/>
+      <c r="B51" s="17"/>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" s="16">
-        <v>0.87000000000000033</v>
-      </c>
-      <c r="B52" s="17">
-        <v>0</v>
-      </c>
+      <c r="A52" s="16"/>
+      <c r="B52" s="17"/>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" s="16">
-        <v>0.88000000000000034</v>
-      </c>
-      <c r="B53" s="17">
-        <v>0</v>
-      </c>
+      <c r="A53" s="16"/>
+      <c r="B53" s="17"/>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A54" s="16">
-        <v>0.89000000000000035</v>
-      </c>
-      <c r="B54" s="17">
-        <v>0</v>
-      </c>
+      <c r="A54" s="16"/>
+      <c r="B54" s="17"/>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A55" s="16">
-        <v>0.90000000000000036</v>
-      </c>
-      <c r="B55" s="17">
-        <v>0</v>
-      </c>
+      <c r="A55" s="16"/>
+      <c r="B55" s="17"/>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A56" s="16">
-        <v>0.91000000000000036</v>
-      </c>
-      <c r="B56" s="17">
-        <v>0</v>
-      </c>
+      <c r="A56" s="16"/>
+      <c r="B56" s="17"/>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A57" s="16">
-        <v>0.92000000000000037</v>
-      </c>
-      <c r="B57" s="17">
-        <v>0</v>
-      </c>
+      <c r="A57" s="16"/>
+      <c r="B57" s="17"/>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A58" s="16">
-        <v>0.93000000000000038</v>
-      </c>
-      <c r="B58" s="17">
-        <v>0</v>
-      </c>
+      <c r="A58" s="16"/>
+      <c r="B58" s="17"/>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59" s="16">
-        <v>0.94000000000000039</v>
-      </c>
-      <c r="B59" s="17">
-        <v>0</v>
-      </c>
+      <c r="A59" s="16"/>
+      <c r="B59" s="17"/>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" s="16">
-        <v>0.9500000000000004</v>
-      </c>
-      <c r="B60" s="17">
-        <v>0</v>
-      </c>
+      <c r="A60" s="16"/>
+      <c r="B60" s="17"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D17:H17"/>
+  </mergeCells>
   <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7" xr:uid="{9887C3D9-0565-4471-929F-C8627F7789A8}">
       <formula1>"n-heptano, n-pentano"</formula1>
@@ -7675,6 +7826,408 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CF99C0D-B9B7-4851-BE57-EA3A1C500665}">
+  <dimension ref="A1:H52"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="15.6640625" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="4">
+        <v>23.1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="5">
+        <v>41.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="5">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="6">
+        <v>15.3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="14">
+        <f>23+273.15</f>
+        <v>296.14999999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="27">
+        <v>0.50725668750098696</v>
+      </c>
+      <c r="B9" s="27">
+        <v>6.5573773225618198E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="27">
+        <v>0.52106194675925599</v>
+      </c>
+      <c r="B10" s="27">
+        <v>7.5409689123005002E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="27">
+        <v>0.536991148148103</v>
+      </c>
+      <c r="B11" s="27">
+        <v>9.8360534766381204E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="27">
+        <v>0.55398228009218398</v>
+      </c>
+      <c r="B12" s="27">
+        <v>1.3114742137919E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="27">
+        <v>0.56778762037056096</v>
+      </c>
+      <c r="B13" s="27">
+        <v>1.6393430799199901E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="27">
+        <v>0.58159296064893795</v>
+      </c>
+      <c r="B14" s="27">
+        <v>1.9999995830931701E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="27">
+        <v>0.59433628935197202</v>
+      </c>
+      <c r="B15" s="27">
+        <v>2.42622635747466E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="27">
+        <v>0.60495575694453696</v>
+      </c>
+      <c r="B16" s="27">
+        <v>2.8524581347380201E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="27">
+        <v>0.61769908564757103</v>
+      </c>
+      <c r="B17" s="27">
+        <v>3.37704907097525E-2</v>
+      </c>
+      <c r="D17" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="27">
+        <v>0.62725662268490101</v>
+      </c>
+      <c r="B18" s="27">
+        <v>3.8032783467976797E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="27">
+        <v>0.641061962963278</v>
+      </c>
+      <c r="B19" s="27">
+        <v>4.4262284420087797E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="27">
+        <v>0.652743361111077</v>
+      </c>
+      <c r="B20" s="27">
+        <v>5.0163921508952498E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="27">
+        <v>0.66442475925887601</v>
+      </c>
+      <c r="B21" s="27">
+        <v>5.5409805856915399E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" s="27">
+        <v>0.67292036574097103</v>
+      </c>
+      <c r="B22" s="27">
+        <v>6.0327863863246199E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" s="27">
+        <v>0.68566369444400499</v>
+      </c>
+      <c r="B23" s="27">
+        <v>6.6229500952110901E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" s="27">
+        <v>0.69840710416714702</v>
+      </c>
+      <c r="B24" s="27">
+        <v>7.1803274177729401E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" s="27">
+        <v>0.71008850231494602</v>
+      </c>
+      <c r="B25" s="27">
+        <v>7.8032787637045006E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26" s="27">
+        <v>0.72070796990751096</v>
+      </c>
+      <c r="B26" s="27">
+        <v>8.2950820628966401E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" s="27">
+        <v>0.73132743750007501</v>
+      </c>
+      <c r="B27" s="27">
+        <v>8.7540977250436899E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" s="27">
+        <v>0.74194690509264005</v>
+      </c>
+      <c r="B28" s="27">
+        <v>9.1803270008661203E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29" s="27">
+        <v>0.75362830324043895</v>
+      </c>
+      <c r="B29" s="27">
+        <v>9.6393439137336306E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" s="27">
+        <v>0.76743364351881604</v>
+      </c>
+      <c r="B30" s="27">
+        <v>0.100327868032314</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" s="27">
+        <v>0.775929168980803</v>
+      </c>
+      <c r="B31" s="27">
+        <v>0.103606556693595</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32" s="27">
+        <v>0.79079643981441505</v>
+      </c>
+      <c r="B32" s="27">
+        <v>0.108196713315065</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" s="27">
+        <v>0.805663710648027</v>
+      </c>
+      <c r="B33" s="27">
+        <v>0.112131142210043</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" s="27">
+        <v>0.82265484259210797</v>
+      </c>
+      <c r="B34" s="27">
+        <v>0.115737700988173</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" s="27">
+        <v>0.83964597453619005</v>
+      </c>
+      <c r="B35" s="27">
+        <v>0.119344259766302</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" s="27">
+        <v>0.85982297916608397</v>
+      </c>
+      <c r="B36" s="27">
+        <v>0.12229507831073499</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" s="27">
+        <v>0.87893805324074303</v>
+      </c>
+      <c r="B37" s="27">
+        <v>0.124918032991921</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" s="27">
+        <v>0.90017698842587202</v>
+      </c>
+      <c r="B38" s="27">
+        <v>0.12590163708886401</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" s="27">
+        <v>0.91823005092518795</v>
+      </c>
+      <c r="B39" s="27">
+        <v>0.12688524743940999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" s="27">
+        <v>0.93522118286927003</v>
+      </c>
+      <c r="B40" s="27">
+        <v>0.126557377322561</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" s="27">
+        <v>0.95115038425811704</v>
+      </c>
+      <c r="B41" s="27">
+        <v>0.124918032991921</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" s="16"/>
+      <c r="B42" s="17"/>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" s="16"/>
+      <c r="B43" s="17"/>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" s="16"/>
+      <c r="B44" s="17"/>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" s="16"/>
+      <c r="B45" s="17"/>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" s="16"/>
+      <c r="B46" s="17"/>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" s="16"/>
+      <c r="B47" s="17"/>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" s="16"/>
+      <c r="B48" s="17"/>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" s="16"/>
+      <c r="B49" s="17"/>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="16"/>
+      <c r="B50" s="17"/>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="16"/>
+      <c r="B51" s="17"/>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="16"/>
+      <c r="B52" s="17"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D17:H17"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7" xr:uid="{8310692E-EC9A-4885-85E2-F4369B6C60C1}">
+      <formula1>"n-heptano, n-pentano"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7977,13 +8530,13 @@
       <c r="B18" s="22">
         <v>1.0418602841124299E-2</v>
       </c>
-      <c r="D18" s="26" t="s">
+      <c r="D18" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -8074,101 +8627,101 @@
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="27">
+      <c r="A9" s="26">
         <v>0.39937236000501602</v>
       </c>
-      <c r="B9" s="27">
+      <c r="B9" s="26">
         <v>4.8785133091925901E-3</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="27">
+      <c r="A10" s="26">
         <v>0.451255237427102</v>
       </c>
-      <c r="B10" s="27">
+      <c r="B10" s="26">
         <v>4.54206345160201E-3</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="27">
+      <c r="A11" s="26">
         <v>0.499790758293094</v>
       </c>
-      <c r="B11" s="27">
+      <c r="B11" s="26">
         <v>4.0373918738397596E-3</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="27">
+      <c r="A12" s="26">
         <v>0.54999995743713403</v>
       </c>
-      <c r="B12" s="27">
+      <c r="B12" s="26">
         <v>3.8691637364208298E-3</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="27">
+      <c r="A13" s="26">
         <v>0.60020915658117302</v>
       </c>
-      <c r="B13" s="27">
+      <c r="B13" s="26">
         <v>1.2616815113045099E-2</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" s="27">
+      <c r="A14" s="26">
         <v>0.64958154850833905</v>
       </c>
-      <c r="B14" s="27">
+      <c r="B14" s="26">
         <v>2.6579442490947201E-2</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="27">
+      <c r="A15" s="26">
         <v>0.69979074765237803</v>
       </c>
-      <c r="B15" s="27">
+      <c r="B15" s="26">
         <v>4.3738321055594401E-2</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="27">
+      <c r="A16" s="26">
         <v>0.751673625074464</v>
       </c>
-      <c r="B16" s="27">
+      <c r="B16" s="26">
         <v>5.9551403398502803E-2</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="27">
+      <c r="A17" s="26">
         <v>0.800209145940457</v>
       </c>
-      <c r="B17" s="27">
+      <c r="B17" s="26">
         <v>7.1327103493442401E-2</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="27">
+      <c r="A18" s="26">
         <v>0.85041834508449698</v>
       </c>
-      <c r="B18" s="27">
+      <c r="B18" s="26">
         <v>7.8897196411617895E-2</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="27">
+      <c r="A19" s="26">
         <v>0.90062754422853597</v>
       </c>
-      <c r="B19" s="27">
+      <c r="B19" s="26">
         <v>8.4953272992194795E-2</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -8346,13 +8899,13 @@
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B32" s="25"/>
@@ -8542,13 +9095,13 @@
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B33" s="25"/>
@@ -8735,13 +9288,13 @@
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B35" s="25"/>
@@ -8922,13 +9475,13 @@
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B33" s="25"/>
@@ -9115,13 +9668,13 @@
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B33" s="25"/>

</xml_diff>

<commit_message>
Parte 1 do Módulo de Cinética de Precipitação. Gráficos de Cinética de Precipitação. Ainda falta a regressão dos dados de cinética a partir dos dados de equilíbrio (experimentais).
</commit_message>
<xml_diff>
--- a/Código_Pré_Modificações_Fred/dados_experimentais.xlsx
+++ b/Código_Pré_Modificações_Fred/dados_experimentais.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vitor\OneDrive\Documentos\Vitor\Projetos\PycharmProjects\Projeto_TotalEnergies\Código_Pré_Modificações_Fred\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC30955E-0E3E-4FEE-B21E-BE89E0251DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{748D41C7-8D0E-4254-8E5E-E53BD16D43BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="12" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Yanes_P1" sheetId="4" r:id="rId1"/>
@@ -7263,74 +7263,74 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="27">
-        <v>0.50725668750098696</v>
+        <v>0</v>
       </c>
       <c r="B9" s="27">
-        <v>3.2786886612808999E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="27">
-        <v>0.53805307870333796</v>
+        <v>0.50725668750098696</v>
       </c>
       <c r="B10" s="27">
-        <v>5.2458968551676198E-3</v>
+        <v>3.2786886612808999E-3</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="27">
-        <v>0.57840708796312601</v>
+        <v>0.53805307870333796</v>
       </c>
       <c r="B11" s="27">
-        <v>2.2622919244106199E-2</v>
+        <v>5.2458968551676198E-3</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="27">
-        <v>0.67185843518573596</v>
+        <v>0.57840708796312601</v>
       </c>
       <c r="B12" s="27">
-        <v>6.7868845282751306E-2</v>
+        <v>2.2622919244106199E-2</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="27">
-        <v>0.70371683796342999</v>
+        <v>0.67185843518573596</v>
       </c>
       <c r="B13" s="27">
-        <v>8.0655736064628794E-2</v>
+        <v>6.7868845282751306E-2</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="27">
-        <v>0.73345129861054503</v>
+        <v>0.70371683796342999</v>
       </c>
       <c r="B14" s="27">
-        <v>9.4426230943449693E-2</v>
+        <v>8.0655736064628794E-2</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="27">
-        <v>0.77380530787033297</v>
+        <v>0.73345129861054503</v>
       </c>
       <c r="B15" s="27">
-        <v>0.10163933599250401</v>
+        <v>9.4426230943449693E-2</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="27">
-        <v>0.87256630786911804</v>
+        <v>0.77380530787033297</v>
       </c>
       <c r="B16" s="27">
-        <v>0.12327868866128</v>
+        <v>0.10163933599250401</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="27">
-        <v>0.93203539120356504</v>
+        <v>0.87256630786911804</v>
       </c>
       <c r="B17" s="27">
-        <v>0.123606558778129</v>
+        <v>0.12327868866128</v>
       </c>
       <c r="D17" s="28" t="s">
         <v>12</v>
@@ -7342,9 +7342,17 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="27">
+        <v>0.93203539120356504</v>
+      </c>
+      <c r="B18" s="27">
+        <v>0.123606558778129</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="27">
         <v>0.95433625694392898</v>
       </c>
-      <c r="B18" s="27">
+      <c r="B19" s="27">
         <v>0.129508183359789</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Parte 2 do Módulo de Cinética de Precipitação. Regressão do modelo cinético a partir dos dados experimentais. Regressão ao longo do tempo ainda não ocorre pois não temos dados ao longo do tempo.
</commit_message>
<xml_diff>
--- a/Código_Pré_Modificações_Fred/dados_experimentais.xlsx
+++ b/Código_Pré_Modificações_Fred/dados_experimentais.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vitor\OneDrive\Documentos\Vitor\Projetos\PycharmProjects\Projeto_TotalEnergies\Código_Pré_Modificações_Fred\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{748D41C7-8D0E-4254-8E5E-E53BD16D43BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9C3D30D-74E7-4F1D-B2A3-25AE489289EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Yanes_P1" sheetId="4" r:id="rId1"/>
@@ -7263,74 +7263,74 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="27">
-        <v>0</v>
+        <v>0.50725668750098696</v>
       </c>
       <c r="B9" s="27">
-        <v>0</v>
+        <v>3.2786886612808999E-3</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="27">
-        <v>0.50725668750098696</v>
+        <v>0.53805307870333796</v>
       </c>
       <c r="B10" s="27">
-        <v>3.2786886612808999E-3</v>
+        <v>5.2458968551676198E-3</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="27">
-        <v>0.53805307870333796</v>
+        <v>0.57840708796312601</v>
       </c>
       <c r="B11" s="27">
-        <v>5.2458968551676198E-3</v>
+        <v>2.2622919244106199E-2</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="27">
-        <v>0.57840708796312601</v>
+        <v>0.67185843518573596</v>
       </c>
       <c r="B12" s="27">
-        <v>2.2622919244106199E-2</v>
+        <v>6.7868845282751306E-2</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="27">
-        <v>0.67185843518573596</v>
+        <v>0.70371683796342999</v>
       </c>
       <c r="B13" s="27">
-        <v>6.7868845282751306E-2</v>
+        <v>8.0655736064628794E-2</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="27">
-        <v>0.70371683796342999</v>
+        <v>0.73345129861054503</v>
       </c>
       <c r="B14" s="27">
-        <v>8.0655736064628794E-2</v>
+        <v>9.4426230943449693E-2</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="27">
-        <v>0.73345129861054503</v>
+        <v>0.77380530787033297</v>
       </c>
       <c r="B15" s="27">
-        <v>9.4426230943449693E-2</v>
+        <v>0.10163933599250401</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="27">
-        <v>0.77380530787033297</v>
+        <v>0.87256630786911804</v>
       </c>
       <c r="B16" s="27">
-        <v>0.10163933599250401</v>
+        <v>0.12327868866128</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="27">
-        <v>0.87256630786911804</v>
+        <v>0.93203539120356504</v>
       </c>
       <c r="B17" s="27">
-        <v>0.12327868866128</v>
+        <v>0.123606558778129</v>
       </c>
       <c r="D17" s="28" t="s">
         <v>12</v>
@@ -7342,17 +7342,9 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="27">
-        <v>0.93203539120356504</v>
+        <v>0.95433625694392898</v>
       </c>
       <c r="B18" s="27">
-        <v>0.123606558778129</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="27">
-        <v>0.95433625694392898</v>
-      </c>
-      <c r="B19" s="27">
         <v>0.129508183359789</v>
       </c>
     </row>

</xml_diff>